<commit_message>
atualização do setor de tecnologia com os dados do 1Q26
</commit_message>
<xml_diff>
--- a/analise_eua/tecnologia/amazon/amzn_indicators.xlsx
+++ b/analise_eua/tecnologia/amazon/amzn_indicators.xlsx
@@ -21,13 +21,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +41,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,13 +49,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,149 +436,149 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="B2" t="n">
@@ -653,7 +667,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="B3" t="n">
@@ -742,7 +756,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>2023</v>
       </c>
       <c r="B4" t="n">
@@ -831,7 +845,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="B5" t="n">
@@ -920,7 +934,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>2021</v>
       </c>
       <c r="B6" t="n">
@@ -1009,7 +1023,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="B7" t="n">
@@ -1098,7 +1112,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>2019</v>
       </c>
       <c r="B8" t="n">
@@ -1187,7 +1201,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="B9" t="n">
@@ -1276,7 +1290,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>2017</v>
       </c>
       <c r="B10" t="n">
@@ -1375,1483 +1389,1572 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC16"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>P/L Damodaran</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>P/L</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>L/P</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Margem Líquida</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>P/VPA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Valor de Mercado</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Dívida Bruta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Caixa e Equivalentes</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/EBITDA</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Dívida Líquida/PL</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>EV/EBITDA</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ROE</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>ROIC</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>FCO</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>FCI</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>FCF</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Free Cash Flow</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Capex</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Net Capex</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Adj Net Capex</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Working Capital</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reinvestment Rate</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>FCFE</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>FCFF</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Buyback</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>45930</v>
+      <c r="A2" s="2" t="n">
+        <v>46112</v>
       </c>
       <c r="B2" t="n">
-        <v>110.62</v>
+        <v>73.95</v>
       </c>
       <c r="C2" t="n">
-        <v>32.43</v>
+        <v>25.62</v>
       </c>
       <c r="D2" t="n">
-        <v>3.08</v>
+        <v>3.9</v>
       </c>
       <c r="E2" t="n">
-        <v>18991</v>
+        <v>42797</v>
       </c>
       <c r="F2" t="n">
-        <v>11.76</v>
+        <v>16.67</v>
       </c>
       <c r="G2" t="n">
-        <v>6.34</v>
+        <v>5.06</v>
       </c>
       <c r="H2" t="n">
-        <v>2343690180</v>
+        <v>2237444610</v>
       </c>
       <c r="I2" t="n">
-        <v>152737</v>
+        <v>224018.832</v>
       </c>
       <c r="J2" t="n">
-        <v>94197</v>
+        <v>143089</v>
       </c>
       <c r="K2" t="n">
-        <v>58540</v>
+        <v>80929.83199999999</v>
       </c>
       <c r="L2" t="n">
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="M2" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="N2" t="n">
-        <v>26.51</v>
+        <v>20.23</v>
       </c>
       <c r="O2" t="n">
-        <v>19.43</v>
+        <v>19.63</v>
       </c>
       <c r="P2" t="n">
-        <v>10.64</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="Q2" t="n">
-        <v>3010</v>
+        <v>26032</v>
       </c>
       <c r="R2" t="n">
-        <v>13351</v>
+        <v>-64212</v>
       </c>
       <c r="S2" t="n">
-        <v>2495</v>
+        <v>52767</v>
       </c>
       <c r="T2" t="n">
-        <v>98</v>
+        <v>-18171</v>
       </c>
       <c r="U2" t="n">
-        <v>2912</v>
+        <v>44203</v>
       </c>
       <c r="V2" t="n">
-        <v>21895</v>
+        <v>43557</v>
       </c>
       <c r="W2" t="n">
-        <v>28962</v>
+        <v>29567</v>
       </c>
       <c r="X2" t="n">
-        <v>123262</v>
+        <v>152246</v>
       </c>
       <c r="Y2" t="n">
-        <v>1670</v>
+        <v>38399</v>
       </c>
       <c r="Z2" t="n">
-        <v>205.72</v>
+        <v>297.04</v>
       </c>
       <c r="AA2" t="n">
-        <v>60558</v>
+        <v>84331</v>
       </c>
       <c r="AB2" t="n">
-        <v>41711</v>
+        <v>4801</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45838</v>
+      <c r="A3" s="2" t="n">
+        <v>45930</v>
       </c>
       <c r="B3" t="n">
-        <v>128.48</v>
+        <v>110.62</v>
       </c>
       <c r="C3" t="n">
-        <v>36.08</v>
+        <v>32.43</v>
       </c>
       <c r="D3" t="n">
-        <v>2.77</v>
+        <v>3.08</v>
       </c>
       <c r="E3" t="n">
-        <v>20136</v>
+        <v>18991</v>
       </c>
       <c r="F3" t="n">
-        <v>10.83</v>
+        <v>11.76</v>
       </c>
       <c r="G3" t="n">
-        <v>6.99</v>
+        <v>6.34</v>
       </c>
       <c r="H3" t="n">
-        <v>2333651430</v>
+        <v>2343690180</v>
       </c>
       <c r="I3" t="n">
-        <v>151917</v>
+        <v>152737</v>
       </c>
       <c r="J3" t="n">
-        <v>93180</v>
+        <v>94197</v>
       </c>
       <c r="K3" t="n">
-        <v>58737</v>
+        <v>58540</v>
       </c>
       <c r="L3" t="n">
-        <v>0.68</v>
+        <v>0.65</v>
       </c>
       <c r="M3" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="N3" t="n">
-        <v>27.61</v>
+        <v>26.51</v>
       </c>
       <c r="O3" t="n">
-        <v>19.21</v>
+        <v>19.43</v>
       </c>
       <c r="P3" t="n">
-        <v>11.93</v>
+        <v>10.64</v>
       </c>
       <c r="Q3" t="n">
-        <v>15500</v>
+        <v>3010</v>
       </c>
       <c r="R3" t="n">
-        <v>-9621</v>
+        <v>13351</v>
       </c>
       <c r="S3" t="n">
-        <v>-2492</v>
+        <v>2495</v>
       </c>
       <c r="T3" t="n">
-        <v>8336</v>
+        <v>98</v>
       </c>
       <c r="U3" t="n">
-        <v>7164</v>
+        <v>2912</v>
       </c>
       <c r="V3" t="n">
-        <v>22893</v>
+        <v>21895</v>
       </c>
       <c r="W3" t="n">
-        <v>27166</v>
+        <v>28962</v>
       </c>
       <c r="X3" t="n">
-        <v>117602</v>
+        <v>123262</v>
       </c>
       <c r="Y3" t="n">
-        <v>4499</v>
+        <v>1670</v>
       </c>
       <c r="Z3" t="n">
-        <v>187.23</v>
+        <v>205.72</v>
       </c>
       <c r="AA3" t="n">
-        <v>46264</v>
+        <v>60558</v>
       </c>
       <c r="AB3" t="n">
-        <v>46916</v>
+        <v>41711</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45747</v>
+      <c r="A4" s="2" t="n">
+        <v>45838</v>
       </c>
       <c r="B4" t="n">
-        <v>117.79</v>
+        <v>128.48</v>
       </c>
       <c r="C4" t="n">
-        <v>35.43</v>
+        <v>36.08</v>
       </c>
       <c r="D4" t="n">
-        <v>2.82</v>
+        <v>2.77</v>
       </c>
       <c r="E4" t="n">
-        <v>32667</v>
+        <v>20136</v>
       </c>
       <c r="F4" t="n">
-        <v>11</v>
+        <v>10.83</v>
       </c>
       <c r="G4" t="n">
-        <v>6.59</v>
+        <v>6.99</v>
       </c>
       <c r="H4" t="n">
-        <v>2017326780</v>
+        <v>2333651430</v>
       </c>
       <c r="I4" t="n">
-        <v>150502</v>
+        <v>151917</v>
       </c>
       <c r="J4" t="n">
-        <v>94565</v>
+        <v>93180</v>
       </c>
       <c r="K4" t="n">
-        <v>55937</v>
+        <v>58737</v>
       </c>
       <c r="L4" t="n">
-        <v>0.6</v>
+        <v>0.68</v>
       </c>
       <c r="M4" t="n">
         <v>0.18</v>
       </c>
       <c r="N4" t="n">
-        <v>22.17</v>
+        <v>27.61</v>
       </c>
       <c r="O4" t="n">
-        <v>18.43</v>
+        <v>19.21</v>
       </c>
       <c r="P4" t="n">
-        <v>11.9</v>
+        <v>11.93</v>
       </c>
       <c r="Q4" t="n">
-        <v>17015</v>
+        <v>15500</v>
       </c>
       <c r="R4" t="n">
-        <v>-29803</v>
+        <v>-9621</v>
       </c>
       <c r="S4" t="n">
-        <v>-47</v>
+        <v>-2492</v>
       </c>
       <c r="T4" t="n">
-        <v>-8004</v>
+        <v>8336</v>
       </c>
       <c r="U4" t="n">
-        <v>25019</v>
+        <v>7164</v>
       </c>
       <c r="V4" t="n">
-        <v>19935</v>
+        <v>22893</v>
       </c>
       <c r="W4" t="n">
-        <v>22994</v>
+        <v>27166</v>
       </c>
       <c r="X4" t="n">
-        <v>107902</v>
+        <v>117602</v>
       </c>
       <c r="Y4" t="n">
-        <v>8474</v>
+        <v>4499</v>
       </c>
       <c r="Z4" t="n">
-        <v>226.78</v>
+        <v>187.23</v>
       </c>
       <c r="AA4" t="n">
-        <v>18385</v>
+        <v>46264</v>
       </c>
       <c r="AB4" t="n">
-        <v>16796</v>
+        <v>46916</v>
       </c>
       <c r="AC4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45565</v>
+      <c r="A5" s="2" t="n">
+        <v>45747</v>
       </c>
       <c r="B5" t="n">
-        <v>127.65</v>
+        <v>117.79</v>
       </c>
       <c r="C5" t="n">
-        <v>39.56</v>
+        <v>35.43</v>
       </c>
       <c r="D5" t="n">
-        <v>2.53</v>
+        <v>2.82</v>
       </c>
       <c r="E5" t="n">
-        <v>18815</v>
+        <v>32667</v>
       </c>
       <c r="F5" t="n">
-        <v>9.65</v>
+        <v>11</v>
       </c>
       <c r="G5" t="n">
-        <v>7.55</v>
+        <v>6.59</v>
       </c>
       <c r="H5" t="n">
-        <v>1956651330</v>
+        <v>2017326780</v>
       </c>
       <c r="I5" t="n">
-        <v>150634</v>
+        <v>150502</v>
       </c>
       <c r="J5" t="n">
-        <v>88051</v>
+        <v>94565</v>
       </c>
       <c r="K5" t="n">
-        <v>62583</v>
+        <v>55937</v>
       </c>
       <c r="L5" t="n">
-        <v>0.86</v>
+        <v>0.6</v>
       </c>
       <c r="M5" t="n">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="N5" t="n">
-        <v>27.83</v>
+        <v>22.17</v>
       </c>
       <c r="O5" t="n">
-        <v>18.96</v>
+        <v>18.43</v>
       </c>
       <c r="P5" t="n">
-        <v>12.04</v>
+        <v>11.9</v>
       </c>
       <c r="Q5" t="n">
-        <v>690</v>
+        <v>17015</v>
       </c>
       <c r="R5" t="n">
-        <v>5239</v>
+        <v>-29803</v>
       </c>
       <c r="S5" t="n">
-        <v>1732</v>
+        <v>-47</v>
       </c>
       <c r="T5" t="n">
-        <v>-4310</v>
+        <v>-8004</v>
       </c>
       <c r="U5" t="n">
-        <v>5000</v>
+        <v>25019</v>
       </c>
       <c r="V5" t="n">
-        <v>9660</v>
+        <v>19935</v>
       </c>
       <c r="W5" t="n">
-        <v>22245</v>
+        <v>22994</v>
       </c>
       <c r="X5" t="n">
-        <v>95836</v>
+        <v>107902</v>
       </c>
       <c r="Y5" t="n">
-        <v>14315</v>
+        <v>8474</v>
       </c>
       <c r="Z5" t="n">
-        <v>196.54</v>
+        <v>226.78</v>
       </c>
       <c r="AA5" t="n">
-        <v>33174</v>
+        <v>18385</v>
       </c>
       <c r="AB5" t="n">
-        <v>39008</v>
+        <v>16796</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>45473</v>
+      <c r="A6" s="2" t="n">
+        <v>45565</v>
       </c>
       <c r="B6" t="n">
-        <v>149.71</v>
+        <v>127.65</v>
       </c>
       <c r="C6" t="n">
-        <v>49.42</v>
+        <v>39.56</v>
       </c>
       <c r="D6" t="n">
-        <v>2.02</v>
+        <v>2.53</v>
       </c>
       <c r="E6" t="n">
-        <v>15026</v>
+        <v>18815</v>
       </c>
       <c r="F6" t="n">
-        <v>9.109999999999999</v>
+        <v>9.65</v>
       </c>
       <c r="G6" t="n">
-        <v>8.539999999999999</v>
+        <v>7.55</v>
       </c>
       <c r="H6" t="n">
-        <v>2018882750</v>
+        <v>1956651330</v>
       </c>
       <c r="I6" t="n">
-        <v>150577</v>
+        <v>150634</v>
       </c>
       <c r="J6" t="n">
-        <v>89092</v>
+        <v>88051</v>
       </c>
       <c r="K6" t="n">
-        <v>61485</v>
+        <v>62583</v>
       </c>
       <c r="L6" t="n">
-        <v>0.99</v>
+        <v>0.86</v>
       </c>
       <c r="M6" t="n">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="N6" t="n">
-        <v>33.61</v>
+        <v>27.83</v>
       </c>
       <c r="O6" t="n">
-        <v>17.15</v>
+        <v>18.96</v>
       </c>
       <c r="P6" t="n">
-        <v>10.72</v>
+        <v>12.04</v>
       </c>
       <c r="Q6" t="n">
-        <v>6292</v>
+        <v>690</v>
       </c>
       <c r="R6" t="n">
-        <v>-4276</v>
+        <v>5239</v>
       </c>
       <c r="S6" t="n">
-        <v>-3234</v>
+        <v>1732</v>
       </c>
       <c r="T6" t="n">
-        <v>3597</v>
+        <v>-4310</v>
       </c>
       <c r="U6" t="n">
-        <v>2695</v>
+        <v>5000</v>
       </c>
       <c r="V6" t="n">
-        <v>2846</v>
+        <v>9660</v>
       </c>
       <c r="W6" t="n">
-        <v>22304</v>
+        <v>22245</v>
       </c>
       <c r="X6" t="n">
-        <v>88708</v>
+        <v>95836</v>
       </c>
       <c r="Y6" t="n">
-        <v>15135</v>
+        <v>14315</v>
       </c>
       <c r="Z6" t="n">
-        <v>204.21</v>
+        <v>196.54</v>
       </c>
       <c r="AA6" t="n">
-        <v>21859</v>
+        <v>33174</v>
       </c>
       <c r="AB6" t="n">
-        <v>44292</v>
+        <v>39008</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45382</v>
+      <c r="A7" s="2" t="n">
+        <v>45473</v>
       </c>
       <c r="B7" t="n">
-        <v>179.72</v>
+        <v>149.71</v>
       </c>
       <c r="C7" t="n">
-        <v>61.56</v>
+        <v>49.42</v>
       </c>
       <c r="D7" t="n">
-        <v>1.62</v>
+        <v>2.02</v>
       </c>
       <c r="E7" t="n">
-        <v>26991</v>
+        <v>15026</v>
       </c>
       <c r="F7" t="n">
-        <v>7.28</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>8.65</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>1874689340</v>
+        <v>2018882750</v>
       </c>
       <c r="I7" t="n">
-        <v>153741</v>
+        <v>150577</v>
       </c>
       <c r="J7" t="n">
-        <v>85074</v>
+        <v>89092</v>
       </c>
       <c r="K7" t="n">
-        <v>68667</v>
+        <v>61485</v>
       </c>
       <c r="L7" t="n">
-        <v>1.09</v>
+        <v>0.99</v>
       </c>
       <c r="M7" t="n">
-        <v>0.32</v>
+        <v>0.26</v>
       </c>
       <c r="N7" t="n">
-        <v>30.96</v>
+        <v>33.61</v>
       </c>
       <c r="O7" t="n">
-        <v>13.95</v>
+        <v>17.15</v>
       </c>
       <c r="P7" t="n">
-        <v>8.75</v>
+        <v>10.72</v>
       </c>
       <c r="Q7" t="n">
-        <v>18989</v>
+        <v>6292</v>
       </c>
       <c r="R7" t="n">
-        <v>-17862</v>
+        <v>-4276</v>
       </c>
       <c r="S7" t="n">
-        <v>-1256</v>
+        <v>-3234</v>
       </c>
       <c r="T7" t="n">
-        <v>4064</v>
+        <v>3597</v>
       </c>
       <c r="U7" t="n">
-        <v>14925</v>
+        <v>2695</v>
       </c>
       <c r="V7" t="n">
-        <v>3589</v>
+        <v>2846</v>
       </c>
       <c r="W7" t="n">
-        <v>20424</v>
+        <v>22304</v>
       </c>
       <c r="X7" t="n">
-        <v>87597</v>
+        <v>88708</v>
       </c>
       <c r="Y7" t="n">
-        <v>11024</v>
+        <v>15135</v>
       </c>
       <c r="Z7" t="n">
-        <v>303.53</v>
+        <v>204.21</v>
       </c>
       <c r="AA7" t="n">
-        <v>5618</v>
+        <v>21859</v>
       </c>
       <c r="AB7" t="n">
-        <v>17139</v>
+        <v>44292</v>
       </c>
       <c r="AC7" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45199</v>
+      <c r="A8" s="2" t="n">
+        <v>45382</v>
       </c>
       <c r="B8" t="n">
-        <v>132.82</v>
+        <v>179.72</v>
       </c>
       <c r="C8" t="n">
-        <v>57.52</v>
+        <v>61.56</v>
       </c>
       <c r="D8" t="n">
-        <v>1.74</v>
+        <v>1.62</v>
       </c>
       <c r="E8" t="n">
-        <v>11730</v>
+        <v>26991</v>
       </c>
       <c r="F8" t="n">
-        <v>6.9</v>
+        <v>7.28</v>
       </c>
       <c r="G8" t="n">
-        <v>7.17</v>
+        <v>8.65</v>
       </c>
       <c r="H8" t="n">
-        <v>1312132640</v>
+        <v>1874689340</v>
       </c>
       <c r="I8" t="n">
-        <v>153461</v>
+        <v>153741</v>
       </c>
       <c r="J8" t="n">
-        <v>64169</v>
+        <v>85074</v>
       </c>
       <c r="K8" t="n">
-        <v>89292</v>
+        <v>68667</v>
       </c>
       <c r="L8" t="n">
-        <v>2.29</v>
+        <v>1.09</v>
       </c>
       <c r="M8" t="n">
-        <v>0.49</v>
+        <v>0.32</v>
       </c>
       <c r="N8" t="n">
-        <v>36.02</v>
+        <v>30.96</v>
       </c>
       <c r="O8" t="n">
-        <v>12.39</v>
+        <v>13.95</v>
       </c>
       <c r="P8" t="n">
-        <v>6.55</v>
+        <v>8.75</v>
       </c>
       <c r="Q8" t="n">
-        <v>4741</v>
+        <v>18989</v>
       </c>
       <c r="R8" t="n">
-        <v>-2080</v>
+        <v>-17862</v>
       </c>
       <c r="S8" t="n">
-        <v>-2409</v>
+        <v>-1256</v>
       </c>
       <c r="T8" t="n">
-        <v>3717</v>
+        <v>4064</v>
       </c>
       <c r="U8" t="n">
-        <v>1024</v>
+        <v>14925</v>
       </c>
       <c r="V8" t="n">
-        <v>392</v>
+        <v>3589</v>
       </c>
       <c r="W8" t="n">
-        <v>21203</v>
+        <v>20424</v>
       </c>
       <c r="X8" t="n">
-        <v>83461</v>
+        <v>87597</v>
       </c>
       <c r="Y8" t="n">
-        <v>-2219</v>
+        <v>11024</v>
       </c>
       <c r="Z8" t="n">
-        <v>363.25</v>
+        <v>303.53</v>
       </c>
       <c r="AA8" t="n">
-        <v>11786</v>
+        <v>5618</v>
       </c>
       <c r="AB8" t="n">
-        <v>24222</v>
+        <v>17139</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45107</v>
+      <c r="A9" s="2" t="n">
+        <v>45199</v>
       </c>
       <c r="B9" t="n">
-        <v>198.63</v>
+        <v>132.82</v>
       </c>
       <c r="C9" t="n">
-        <v>124.15</v>
+        <v>57.52</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.74</v>
       </c>
       <c r="E9" t="n">
-        <v>8147</v>
+        <v>11730</v>
       </c>
       <c r="F9" t="n">
-        <v>5.02</v>
+        <v>6.9</v>
       </c>
       <c r="G9" t="n">
-        <v>7.95</v>
+        <v>7.17</v>
       </c>
       <c r="H9" t="n">
-        <v>1340752600</v>
+        <v>1312132640</v>
       </c>
       <c r="I9" t="n">
-        <v>153917</v>
+        <v>153461</v>
       </c>
       <c r="J9" t="n">
-        <v>63970</v>
+        <v>64169</v>
       </c>
       <c r="K9" t="n">
-        <v>89947</v>
+        <v>89292</v>
       </c>
       <c r="L9" t="n">
-        <v>2.89</v>
+        <v>2.29</v>
       </c>
       <c r="M9" t="n">
-        <v>0.53</v>
+        <v>0.49</v>
       </c>
       <c r="N9" t="n">
-        <v>45.99</v>
+        <v>36.02</v>
       </c>
       <c r="O9" t="n">
-        <v>6.39</v>
+        <v>12.39</v>
       </c>
       <c r="P9" t="n">
-        <v>5.31</v>
+        <v>6.55</v>
       </c>
       <c r="Q9" t="n">
-        <v>11688</v>
+        <v>4741</v>
       </c>
       <c r="R9" t="n">
-        <v>6133</v>
+        <v>-2080</v>
       </c>
       <c r="S9" t="n">
-        <v>-12893</v>
+        <v>-2409</v>
       </c>
       <c r="T9" t="n">
-        <v>14440</v>
+        <v>3717</v>
       </c>
       <c r="U9" t="n">
-        <v>-2752</v>
+        <v>1024</v>
       </c>
       <c r="V9" t="n">
-        <v>67</v>
+        <v>392</v>
       </c>
       <c r="W9" t="n">
-        <v>21931</v>
+        <v>21203</v>
       </c>
       <c r="X9" t="n">
-        <v>80005</v>
+        <v>83461</v>
       </c>
       <c r="Y9" t="n">
-        <v>-7756</v>
+        <v>-2219</v>
       </c>
       <c r="Z9" t="n">
-        <v>433.45</v>
+        <v>363.25</v>
       </c>
       <c r="AA9" t="n">
-        <v>8349</v>
+        <v>11786</v>
       </c>
       <c r="AB9" t="n">
-        <v>22114</v>
+        <v>24222</v>
       </c>
       <c r="AC9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>45016</v>
+      <c r="A10" s="2" t="n">
+        <v>45107</v>
       </c>
       <c r="B10" t="n">
-        <v>333.77</v>
+        <v>198.63</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>124.15</v>
       </c>
       <c r="D10" t="n">
-        <v>-6.93</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E10" t="n">
-        <v>15897</v>
+        <v>8147</v>
       </c>
       <c r="F10" t="n">
-        <v>2.49</v>
+        <v>5.02</v>
       </c>
       <c r="G10" t="n">
-        <v>6.85</v>
+        <v>7.95</v>
       </c>
       <c r="H10" t="n">
-        <v>1058722500</v>
+        <v>1340752600</v>
       </c>
       <c r="I10" t="n">
-        <v>154779</v>
+        <v>153917</v>
       </c>
       <c r="J10" t="n">
-        <v>64405</v>
+        <v>63970</v>
       </c>
       <c r="K10" t="n">
-        <v>90374</v>
+        <v>89947</v>
       </c>
       <c r="L10" t="n">
-        <v>2.54</v>
+        <v>2.89</v>
       </c>
       <c r="M10" t="n">
-        <v>0.58</v>
+        <v>0.53</v>
       </c>
       <c r="N10" t="n">
-        <v>32.27</v>
+        <v>45.99</v>
       </c>
       <c r="O10" t="n">
-        <v>0.11</v>
+        <v>6.39</v>
       </c>
       <c r="P10" t="n">
-        <v>4.96</v>
+        <v>5.31</v>
       </c>
       <c r="Q10" t="n">
-        <v>4788</v>
+        <v>11688</v>
       </c>
       <c r="R10" t="n">
-        <v>-15806</v>
+        <v>6133</v>
       </c>
       <c r="S10" t="n">
-        <v>6354</v>
+        <v>-12893</v>
       </c>
       <c r="T10" t="n">
-        <v>-9419</v>
+        <v>14440</v>
       </c>
       <c r="U10" t="n">
-        <v>14207</v>
+        <v>-2752</v>
       </c>
       <c r="V10" t="n">
-        <v>9258</v>
+        <v>67</v>
       </c>
       <c r="W10" t="n">
-        <v>20450</v>
+        <v>21931</v>
       </c>
       <c r="X10" t="n">
-        <v>82107</v>
+        <v>80005</v>
       </c>
       <c r="Y10" t="n">
-        <v>-11349</v>
+        <v>-7756</v>
       </c>
       <c r="Z10" t="n">
-        <v>653.09</v>
+        <v>433.45</v>
       </c>
       <c r="AA10" t="n">
-        <v>-17708</v>
+        <v>8349</v>
       </c>
       <c r="AB10" t="n">
-        <v>-16253</v>
+        <v>22114</v>
       </c>
       <c r="AC10" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>44834</v>
+      <c r="A11" s="2" t="n">
+        <v>45016</v>
       </c>
       <c r="B11" t="n">
-        <v>400.97</v>
+        <v>333.77</v>
       </c>
       <c r="C11" t="n">
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>-1.11</v>
+        <v>-6.93</v>
       </c>
       <c r="E11" t="n">
-        <v>3135</v>
+        <v>15897</v>
       </c>
       <c r="F11" t="n">
-        <v>2.26</v>
+        <v>2.49</v>
       </c>
       <c r="G11" t="n">
-        <v>8.380000000000001</v>
+        <v>6.85</v>
       </c>
       <c r="H11" t="n">
-        <v>1151583000</v>
+        <v>1058722500</v>
       </c>
       <c r="I11" t="n">
-        <v>144580</v>
+        <v>154779</v>
       </c>
       <c r="J11" t="n">
-        <v>58662</v>
+        <v>64405</v>
       </c>
       <c r="K11" t="n">
-        <v>85918</v>
+        <v>90374</v>
       </c>
       <c r="L11" t="n">
-        <v>3.37</v>
+        <v>2.54</v>
       </c>
       <c r="M11" t="n">
-        <v>0.62</v>
+        <v>0.58</v>
       </c>
       <c r="N11" t="n">
-        <v>48.57</v>
+        <v>32.27</v>
       </c>
       <c r="O11" t="n">
         <v>0.11</v>
       </c>
       <c r="P11" t="n">
-        <v>5.39</v>
+        <v>4.96</v>
       </c>
       <c r="Q11" t="n">
-        <v>2439</v>
+        <v>4788</v>
       </c>
       <c r="R11" t="n">
-        <v>-3530</v>
+        <v>-15806</v>
       </c>
       <c r="S11" t="n">
-        <v>-1610</v>
+        <v>6354</v>
       </c>
       <c r="T11" t="n">
-        <v>1785</v>
+        <v>-9419</v>
       </c>
       <c r="U11" t="n">
-        <v>654</v>
+        <v>14207</v>
       </c>
       <c r="V11" t="n">
-        <v>6724</v>
+        <v>9258</v>
       </c>
       <c r="W11" t="n">
-        <v>19485</v>
+        <v>20450</v>
       </c>
       <c r="X11" t="n">
-        <v>73503</v>
+        <v>82107</v>
       </c>
       <c r="Y11" t="n">
-        <v>-8900</v>
+        <v>-11349</v>
       </c>
       <c r="Z11" t="n">
-        <v>457.6</v>
+        <v>653.09</v>
       </c>
       <c r="AA11" t="n">
-        <v>-18014</v>
+        <v>-17708</v>
       </c>
       <c r="AB11" t="n">
-        <v>11259</v>
+        <v>-16253</v>
       </c>
       <c r="AC11" t="n">
-        <v>-3334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>44742</v>
+      <c r="A12" s="2" t="n">
+        <v>44834</v>
       </c>
       <c r="B12" t="n">
-        <v>-532.88</v>
+        <v>400.97</v>
       </c>
       <c r="C12" t="n">
-        <v>7.66</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>13.06</v>
+        <v>-1.11</v>
       </c>
       <c r="E12" t="n">
-        <v>3933</v>
+        <v>3135</v>
       </c>
       <c r="F12" t="n">
-        <v>-1.67</v>
+        <v>2.26</v>
       </c>
       <c r="G12" t="n">
-        <v>8.23</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="H12" t="n">
-        <v>1080686750</v>
+        <v>1151583000</v>
       </c>
       <c r="I12" t="n">
-        <v>142074</v>
+        <v>144580</v>
       </c>
       <c r="J12" t="n">
-        <v>60710</v>
+        <v>58662</v>
       </c>
       <c r="K12" t="n">
-        <v>81364</v>
+        <v>85918</v>
       </c>
       <c r="L12" t="n">
-        <v>2.66</v>
+        <v>3.37</v>
       </c>
       <c r="M12" t="n">
         <v>0.62</v>
       </c>
       <c r="N12" t="n">
-        <v>38.01</v>
+        <v>48.57</v>
       </c>
       <c r="O12" t="n">
-        <v>3.85</v>
+        <v>0.11</v>
       </c>
       <c r="P12" t="n">
-        <v>7.16</v>
+        <v>5.39</v>
       </c>
       <c r="Q12" t="n">
-        <v>11755</v>
+        <v>2439</v>
       </c>
       <c r="R12" t="n">
-        <v>-12984</v>
+        <v>-3530</v>
       </c>
       <c r="S12" t="n">
-        <v>2636</v>
+        <v>-1610</v>
       </c>
       <c r="T12" t="n">
-        <v>10982</v>
+        <v>1785</v>
       </c>
       <c r="U12" t="n">
-        <v>773</v>
+        <v>654</v>
       </c>
       <c r="V12" t="n">
-        <v>8356</v>
+        <v>6724</v>
       </c>
       <c r="W12" t="n">
-        <v>18072</v>
+        <v>19485</v>
       </c>
       <c r="X12" t="n">
-        <v>69521</v>
+        <v>73503</v>
       </c>
       <c r="Y12" t="n">
-        <v>-6624</v>
+        <v>-8900</v>
       </c>
       <c r="Z12" t="n">
-        <v>303.84</v>
+        <v>457.6</v>
       </c>
       <c r="AA12" t="n">
-        <v>15408</v>
+        <v>-18014</v>
       </c>
       <c r="AB12" t="n">
-        <v>16534</v>
+        <v>11259</v>
       </c>
       <c r="AC12" t="n">
-        <v>668</v>
+        <v>-3334</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>44651</v>
+      <c r="A13" s="2" t="n">
+        <v>44742</v>
       </c>
       <c r="B13" t="n">
-        <v>-431.67</v>
+        <v>-532.88</v>
       </c>
       <c r="C13" t="n">
-        <v>108.09</v>
+        <v>7.66</v>
       </c>
       <c r="D13" t="n">
-        <v>0.93</v>
+        <v>13.06</v>
       </c>
       <c r="E13" t="n">
-        <v>12647</v>
+        <v>3933</v>
       </c>
       <c r="F13" t="n">
-        <v>-3.3</v>
+        <v>-1.67</v>
       </c>
       <c r="G13" t="n">
-        <v>12.38</v>
+        <v>8.23</v>
       </c>
       <c r="H13" t="n">
-        <v>1659340000</v>
+        <v>1080686750</v>
       </c>
       <c r="I13" t="n">
-        <v>129450</v>
+        <v>142074</v>
       </c>
       <c r="J13" t="n">
-        <v>66385</v>
+        <v>60710</v>
       </c>
       <c r="K13" t="n">
-        <v>63065</v>
+        <v>81364</v>
       </c>
       <c r="L13" t="n">
-        <v>1.47</v>
+        <v>2.66</v>
       </c>
       <c r="M13" t="n">
-        <v>0.47</v>
+        <v>0.62</v>
       </c>
       <c r="N13" t="n">
-        <v>40.04</v>
+        <v>38.01</v>
       </c>
       <c r="O13" t="n">
-        <v>11.34</v>
+        <v>3.85</v>
       </c>
       <c r="P13" t="n">
-        <v>8.48</v>
+        <v>7.16</v>
       </c>
       <c r="Q13" t="n">
-        <v>-2790</v>
+        <v>11755</v>
       </c>
       <c r="R13" t="n">
-        <v>906</v>
+        <v>-12984</v>
       </c>
       <c r="S13" t="n">
-        <v>1990</v>
+        <v>2636</v>
       </c>
       <c r="T13" t="n">
-        <v>-17741</v>
+        <v>10982</v>
       </c>
       <c r="U13" t="n">
-        <v>14951</v>
+        <v>773</v>
       </c>
       <c r="V13" t="n">
-        <v>12773</v>
+        <v>8356</v>
       </c>
       <c r="W13" t="n">
-        <v>14842</v>
+        <v>18072</v>
       </c>
       <c r="X13" t="n">
-        <v>68354</v>
+        <v>69521</v>
       </c>
       <c r="Y13" t="n">
-        <v>-5632</v>
+        <v>-6624</v>
       </c>
       <c r="Z13" t="n">
-        <v>396.01</v>
+        <v>303.84</v>
       </c>
       <c r="AA13" t="n">
-        <v>-15774</v>
+        <v>15408</v>
       </c>
       <c r="AB13" t="n">
-        <v>-14539</v>
+        <v>16534</v>
       </c>
       <c r="AC13" t="n">
-        <v>2666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>44469</v>
+      <c r="A14" s="2" t="n">
+        <v>44651</v>
       </c>
       <c r="B14" t="n">
-        <v>527.72</v>
+        <v>-431.67</v>
       </c>
       <c r="C14" t="n">
-        <v>65.23999999999999</v>
+        <v>108.09</v>
       </c>
       <c r="D14" t="n">
-        <v>1.53</v>
+        <v>0.93</v>
       </c>
       <c r="E14" t="n">
-        <v>5762</v>
+        <v>12647</v>
       </c>
       <c r="F14" t="n">
-        <v>2.85</v>
+        <v>-3.3</v>
       </c>
       <c r="G14" t="n">
-        <v>13.81</v>
+        <v>12.38</v>
       </c>
       <c r="H14" t="n">
-        <v>1665495000</v>
+        <v>1659340000</v>
       </c>
       <c r="I14" t="n">
-        <v>129528</v>
+        <v>129450</v>
       </c>
       <c r="J14" t="n">
-        <v>78988</v>
+        <v>66385</v>
       </c>
       <c r="K14" t="n">
-        <v>50540</v>
+        <v>63065</v>
       </c>
       <c r="L14" t="n">
-        <v>1.35</v>
+        <v>1.47</v>
       </c>
       <c r="M14" t="n">
-        <v>0.42</v>
+        <v>0.47</v>
       </c>
       <c r="N14" t="n">
-        <v>45.96</v>
+        <v>40.04</v>
       </c>
       <c r="O14" t="n">
-        <v>21.04</v>
+        <v>11.34</v>
       </c>
       <c r="P14" t="n">
-        <v>9.140000000000001</v>
+        <v>8.48</v>
       </c>
       <c r="Q14" t="n">
-        <v>-5402</v>
+        <v>-2790</v>
       </c>
       <c r="R14" t="n">
-        <v>7252</v>
+        <v>906</v>
       </c>
       <c r="S14" t="n">
-        <v>-18419</v>
+        <v>1990</v>
       </c>
       <c r="T14" t="n">
-        <v>-6862</v>
+        <v>-17741</v>
       </c>
       <c r="U14" t="n">
-        <v>1460</v>
+        <v>14951</v>
       </c>
       <c r="V14" t="n">
-        <v>9629</v>
+        <v>12773</v>
       </c>
       <c r="W14" t="n">
-        <v>14380</v>
+        <v>14842</v>
       </c>
       <c r="X14" t="n">
-        <v>61344</v>
+        <v>68354</v>
       </c>
       <c r="Y14" t="n">
-        <v>14537</v>
+        <v>-5632</v>
       </c>
       <c r="Z14" t="n">
-        <v>280.9</v>
+        <v>396.01</v>
       </c>
       <c r="AA14" t="n">
-        <v>-1429</v>
+        <v>-15774</v>
       </c>
       <c r="AB14" t="n">
-        <v>7710</v>
+        <v>-14539</v>
       </c>
       <c r="AC14" t="n">
-        <v>0</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>44377</v>
+      <c r="A15" s="2" t="n">
+        <v>44469</v>
       </c>
       <c r="B15" t="n">
-        <v>223.36</v>
+        <v>527.72</v>
       </c>
       <c r="C15" t="n">
-        <v>62.98</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>1.59</v>
+        <v>1.53</v>
       </c>
       <c r="E15" t="n">
-        <v>8232</v>
+        <v>5762</v>
       </c>
       <c r="F15" t="n">
-        <v>6.88</v>
+        <v>2.85</v>
       </c>
       <c r="G15" t="n">
-        <v>15.13</v>
+        <v>13.81</v>
       </c>
       <c r="H15" t="n">
-        <v>1737301000</v>
+        <v>1665495000</v>
       </c>
       <c r="I15" t="n">
-        <v>122390</v>
+        <v>129528</v>
       </c>
       <c r="J15" t="n">
-        <v>89894</v>
+        <v>78988</v>
       </c>
       <c r="K15" t="n">
-        <v>32496</v>
+        <v>50540</v>
       </c>
       <c r="L15" t="n">
-        <v>0.86</v>
+        <v>1.35</v>
       </c>
       <c r="M15" t="n">
-        <v>0.28</v>
+        <v>0.42</v>
       </c>
       <c r="N15" t="n">
-        <v>46.82</v>
+        <v>45.96</v>
       </c>
       <c r="O15" t="n">
-        <v>23.92</v>
+        <v>21.04</v>
       </c>
       <c r="P15" t="n">
-        <v>10.96</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="Q15" t="n">
-        <v>8502</v>
+        <v>-5402</v>
       </c>
       <c r="R15" t="n">
-        <v>-13414</v>
+        <v>7252</v>
       </c>
       <c r="S15" t="n">
-        <v>19119</v>
+        <v>-18419</v>
       </c>
       <c r="T15" t="n">
-        <v>6296</v>
+        <v>-6862</v>
       </c>
       <c r="U15" t="n">
-        <v>2206</v>
+        <v>1460</v>
       </c>
       <c r="V15" t="n">
-        <v>9357</v>
+        <v>9629</v>
       </c>
       <c r="W15" t="n">
-        <v>13871</v>
+        <v>14380</v>
       </c>
       <c r="X15" t="n">
-        <v>57080</v>
+        <v>61344</v>
       </c>
       <c r="Y15" t="n">
-        <v>23056</v>
+        <v>14537</v>
       </c>
       <c r="Z15" t="n">
-        <v>193.31</v>
+        <v>280.9</v>
       </c>
       <c r="AA15" t="n">
-        <v>38394</v>
+        <v>-1429</v>
       </c>
       <c r="AB15" t="n">
-        <v>23201</v>
+        <v>7710</v>
       </c>
       <c r="AC15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
+        <v>44377</v>
+      </c>
+      <c r="B16" t="n">
+        <v>223.36</v>
+      </c>
+      <c r="C16" t="n">
+        <v>62.98</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="E16" t="n">
+        <v>8232</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="G16" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="H16" t="n">
+        <v>1737301000</v>
+      </c>
+      <c r="I16" t="n">
+        <v>122390</v>
+      </c>
+      <c r="J16" t="n">
+        <v>89894</v>
+      </c>
+      <c r="K16" t="n">
+        <v>32496</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="N16" t="n">
+        <v>46.82</v>
+      </c>
+      <c r="O16" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P16" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>8502</v>
+      </c>
+      <c r="R16" t="n">
+        <v>-13414</v>
+      </c>
+      <c r="S16" t="n">
+        <v>19119</v>
+      </c>
+      <c r="T16" t="n">
+        <v>6296</v>
+      </c>
+      <c r="U16" t="n">
+        <v>2206</v>
+      </c>
+      <c r="V16" t="n">
+        <v>9357</v>
+      </c>
+      <c r="W16" t="n">
+        <v>13871</v>
+      </c>
+      <c r="X16" t="n">
+        <v>57080</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>23056</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="AA16" t="n">
+        <v>38394</v>
+      </c>
+      <c r="AB16" t="n">
+        <v>23201</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>44286</v>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>192.35</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C17" t="n">
         <v>69.83</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D17" t="n">
         <v>1.43</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E17" t="n">
         <v>16373</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F17" t="n">
         <v>7.47</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G17" t="n">
         <v>15.09</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H17" t="n">
         <v>1559376000</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I17" t="n">
         <v>100794</v>
       </c>
-      <c r="J16" t="n">
+      <c r="J17" t="n">
         <v>73270</v>
       </c>
-      <c r="K16" t="n">
+      <c r="K17" t="n">
         <v>27524</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L17" t="n">
         <v>0.71</v>
       </c>
-      <c r="M16" t="n">
+      <c r="M17" t="n">
         <v>0.27</v>
       </c>
-      <c r="N16" t="n">
+      <c r="N17" t="n">
         <v>40.77</v>
       </c>
-      <c r="O16" t="n">
+      <c r="O17" t="n">
         <v>21.5</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P17" t="n">
         <v>10.98</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q17" t="n">
         <v>4213</v>
       </c>
-      <c r="R16" t="n">
+      <c r="R17" t="n">
         <v>-8666</v>
       </c>
-      <c r="S16" t="n">
+      <c r="S17" t="n">
         <v>-3476</v>
       </c>
-      <c r="T16" t="n">
+      <c r="T17" t="n">
         <v>-7869</v>
       </c>
-      <c r="U16" t="n">
+      <c r="U17" t="n">
         <v>12082</v>
       </c>
-      <c r="V16" t="n">
+      <c r="V17" t="n">
         <v>9114</v>
       </c>
-      <c r="W16" t="n">
+      <c r="W17" t="n">
         <v>12488</v>
       </c>
-      <c r="X16" t="n">
+      <c r="X17" t="n">
         <v>52291</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="Y17" t="n">
         <v>6004</v>
       </c>
-      <c r="Z16" t="n">
+      <c r="Z17" t="n">
         <v>288.2</v>
       </c>
-      <c r="AA16" t="n">
+      <c r="AA17" t="n">
         <v>-6761</v>
       </c>
-      <c r="AB16" t="n">
+      <c r="AB17" t="n">
         <v>-1731</v>
       </c>
-      <c r="AC16" t="n">
+      <c r="AC17" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
atualizei os dados do 2Q26 da AMZN
</commit_message>
<xml_diff>
--- a/analise_eua/tecnologia/amazon/amzn_indicators.xlsx
+++ b/analise_eua/tecnologia/amazon/amzn_indicators.xlsx
@@ -1389,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC17"/>
+  <dimension ref="A1:AC18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1536,88 +1536,88 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46112</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="n">
-        <v>73.95</v>
+        <v>40.97</v>
       </c>
       <c r="C2" t="n">
-        <v>25.62</v>
+        <v>19.33</v>
       </c>
       <c r="D2" t="n">
-        <v>3.9</v>
+        <v>5.17</v>
       </c>
       <c r="E2" t="n">
-        <v>42797</v>
+        <v>28504</v>
       </c>
       <c r="F2" t="n">
-        <v>16.67</v>
+        <v>31.23</v>
       </c>
       <c r="G2" t="n">
-        <v>5.06</v>
+        <v>4.65</v>
       </c>
       <c r="H2" t="n">
-        <v>2237444610</v>
+        <v>2566683460</v>
       </c>
       <c r="I2" t="n">
-        <v>224018.832</v>
+        <v>241995</v>
       </c>
       <c r="J2" t="n">
-        <v>143089</v>
+        <v>122988</v>
       </c>
       <c r="K2" t="n">
-        <v>80929.83199999999</v>
+        <v>119007</v>
       </c>
       <c r="L2" t="n">
-        <v>0.71</v>
+        <v>1.08</v>
       </c>
       <c r="M2" t="n">
-        <v>0.18</v>
+        <v>0.22</v>
       </c>
       <c r="N2" t="n">
-        <v>20.23</v>
+        <v>24.32</v>
       </c>
       <c r="O2" t="n">
-        <v>19.63</v>
+        <v>23.98</v>
       </c>
       <c r="P2" t="n">
-        <v>8.279999999999999</v>
+        <v>6.37</v>
       </c>
       <c r="Q2" t="n">
-        <v>26032</v>
+        <v>19355</v>
       </c>
       <c r="R2" t="n">
-        <v>-64212</v>
+        <v>-15033</v>
       </c>
       <c r="S2" t="n">
-        <v>52767</v>
+        <v>-42621</v>
       </c>
       <c r="T2" t="n">
-        <v>-18171</v>
+        <v>9350</v>
       </c>
       <c r="U2" t="n">
-        <v>44203</v>
+        <v>10005</v>
       </c>
       <c r="V2" t="n">
-        <v>43557</v>
+        <v>41762</v>
       </c>
       <c r="W2" t="n">
-        <v>29567</v>
+        <v>33158</v>
       </c>
       <c r="X2" t="n">
-        <v>152246</v>
+        <v>160615</v>
       </c>
       <c r="Y2" t="n">
-        <v>38399</v>
+        <v>7990</v>
       </c>
       <c r="Z2" t="n">
-        <v>297.04</v>
+        <v>274.83</v>
       </c>
       <c r="AA2" t="n">
-        <v>84331</v>
+        <v>122303</v>
       </c>
       <c r="AB2" t="n">
-        <v>4801</v>
+        <v>48021</v>
       </c>
       <c r="AC2" t="n">
         <v>0</v>
@@ -1625,88 +1625,88 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45930</v>
+        <v>46112</v>
       </c>
       <c r="B3" t="n">
-        <v>110.62</v>
+        <v>73.95</v>
       </c>
       <c r="C3" t="n">
-        <v>32.43</v>
+        <v>25.62</v>
       </c>
       <c r="D3" t="n">
-        <v>3.08</v>
+        <v>3.9</v>
       </c>
       <c r="E3" t="n">
-        <v>18991</v>
+        <v>42797</v>
       </c>
       <c r="F3" t="n">
-        <v>11.76</v>
+        <v>16.67</v>
       </c>
       <c r="G3" t="n">
-        <v>6.34</v>
+        <v>5.06</v>
       </c>
       <c r="H3" t="n">
-        <v>2343690180</v>
+        <v>2237444610</v>
       </c>
       <c r="I3" t="n">
-        <v>152737</v>
+        <v>224018.832</v>
       </c>
       <c r="J3" t="n">
-        <v>94197</v>
+        <v>143089</v>
       </c>
       <c r="K3" t="n">
-        <v>58540</v>
+        <v>80929.83199999999</v>
       </c>
       <c r="L3" t="n">
-        <v>0.65</v>
+        <v>0.71</v>
       </c>
       <c r="M3" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="N3" t="n">
-        <v>26.51</v>
+        <v>20.23</v>
       </c>
       <c r="O3" t="n">
-        <v>19.43</v>
+        <v>19.63</v>
       </c>
       <c r="P3" t="n">
-        <v>10.64</v>
+        <v>8.279999999999999</v>
       </c>
       <c r="Q3" t="n">
-        <v>3010</v>
+        <v>26032</v>
       </c>
       <c r="R3" t="n">
-        <v>13351</v>
+        <v>-64212</v>
       </c>
       <c r="S3" t="n">
-        <v>2495</v>
+        <v>52767</v>
       </c>
       <c r="T3" t="n">
-        <v>98</v>
+        <v>-18171</v>
       </c>
       <c r="U3" t="n">
-        <v>2912</v>
+        <v>44203</v>
       </c>
       <c r="V3" t="n">
-        <v>21895</v>
+        <v>43557</v>
       </c>
       <c r="W3" t="n">
-        <v>28962</v>
+        <v>29567</v>
       </c>
       <c r="X3" t="n">
-        <v>123262</v>
+        <v>152246</v>
       </c>
       <c r="Y3" t="n">
-        <v>1670</v>
+        <v>38399</v>
       </c>
       <c r="Z3" t="n">
-        <v>205.72</v>
+        <v>297.04</v>
       </c>
       <c r="AA3" t="n">
-        <v>60558</v>
+        <v>84331</v>
       </c>
       <c r="AB3" t="n">
-        <v>41711</v>
+        <v>4801</v>
       </c>
       <c r="AC3" t="n">
         <v>0</v>
@@ -1714,88 +1714,88 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45838</v>
+        <v>45930</v>
       </c>
       <c r="B4" t="n">
-        <v>128.48</v>
+        <v>110.62</v>
       </c>
       <c r="C4" t="n">
-        <v>36.08</v>
+        <v>32.43</v>
       </c>
       <c r="D4" t="n">
-        <v>2.77</v>
+        <v>3.08</v>
       </c>
       <c r="E4" t="n">
-        <v>20136</v>
+        <v>18991</v>
       </c>
       <c r="F4" t="n">
-        <v>10.83</v>
+        <v>11.76</v>
       </c>
       <c r="G4" t="n">
-        <v>6.99</v>
+        <v>6.34</v>
       </c>
       <c r="H4" t="n">
-        <v>2333651430</v>
+        <v>2343690180</v>
       </c>
       <c r="I4" t="n">
-        <v>151917</v>
+        <v>152737</v>
       </c>
       <c r="J4" t="n">
-        <v>93180</v>
+        <v>94197</v>
       </c>
       <c r="K4" t="n">
-        <v>58737</v>
+        <v>58540</v>
       </c>
       <c r="L4" t="n">
-        <v>0.68</v>
+        <v>0.65</v>
       </c>
       <c r="M4" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="N4" t="n">
-        <v>27.61</v>
+        <v>26.51</v>
       </c>
       <c r="O4" t="n">
-        <v>19.21</v>
+        <v>19.43</v>
       </c>
       <c r="P4" t="n">
-        <v>11.93</v>
+        <v>10.64</v>
       </c>
       <c r="Q4" t="n">
-        <v>15500</v>
+        <v>3010</v>
       </c>
       <c r="R4" t="n">
-        <v>-9621</v>
+        <v>13351</v>
       </c>
       <c r="S4" t="n">
-        <v>-2492</v>
+        <v>2495</v>
       </c>
       <c r="T4" t="n">
-        <v>8336</v>
+        <v>98</v>
       </c>
       <c r="U4" t="n">
-        <v>7164</v>
+        <v>2912</v>
       </c>
       <c r="V4" t="n">
-        <v>22893</v>
+        <v>21895</v>
       </c>
       <c r="W4" t="n">
-        <v>27166</v>
+        <v>28962</v>
       </c>
       <c r="X4" t="n">
-        <v>117602</v>
+        <v>123262</v>
       </c>
       <c r="Y4" t="n">
-        <v>4499</v>
+        <v>1670</v>
       </c>
       <c r="Z4" t="n">
-        <v>187.23</v>
+        <v>205.72</v>
       </c>
       <c r="AA4" t="n">
-        <v>46264</v>
+        <v>60558</v>
       </c>
       <c r="AB4" t="n">
-        <v>46916</v>
+        <v>41711</v>
       </c>
       <c r="AC4" t="n">
         <v>0</v>
@@ -1803,88 +1803,88 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45747</v>
+        <v>45838</v>
       </c>
       <c r="B5" t="n">
-        <v>117.79</v>
+        <v>128.48</v>
       </c>
       <c r="C5" t="n">
-        <v>35.43</v>
+        <v>36.08</v>
       </c>
       <c r="D5" t="n">
-        <v>2.82</v>
+        <v>2.77</v>
       </c>
       <c r="E5" t="n">
-        <v>32667</v>
+        <v>20136</v>
       </c>
       <c r="F5" t="n">
-        <v>11</v>
+        <v>10.83</v>
       </c>
       <c r="G5" t="n">
-        <v>6.59</v>
+        <v>6.99</v>
       </c>
       <c r="H5" t="n">
-        <v>2017326780</v>
+        <v>2333651430</v>
       </c>
       <c r="I5" t="n">
-        <v>150502</v>
+        <v>151917</v>
       </c>
       <c r="J5" t="n">
-        <v>94565</v>
+        <v>93180</v>
       </c>
       <c r="K5" t="n">
-        <v>55937</v>
+        <v>58737</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6</v>
+        <v>0.68</v>
       </c>
       <c r="M5" t="n">
         <v>0.18</v>
       </c>
       <c r="N5" t="n">
-        <v>22.17</v>
+        <v>27.61</v>
       </c>
       <c r="O5" t="n">
-        <v>18.43</v>
+        <v>19.21</v>
       </c>
       <c r="P5" t="n">
-        <v>11.9</v>
+        <v>11.93</v>
       </c>
       <c r="Q5" t="n">
-        <v>17015</v>
+        <v>15500</v>
       </c>
       <c r="R5" t="n">
-        <v>-29803</v>
+        <v>-9621</v>
       </c>
       <c r="S5" t="n">
-        <v>-47</v>
+        <v>-2492</v>
       </c>
       <c r="T5" t="n">
-        <v>-8004</v>
+        <v>8336</v>
       </c>
       <c r="U5" t="n">
-        <v>25019</v>
+        <v>7164</v>
       </c>
       <c r="V5" t="n">
-        <v>19935</v>
+        <v>22893</v>
       </c>
       <c r="W5" t="n">
-        <v>22994</v>
+        <v>27166</v>
       </c>
       <c r="X5" t="n">
-        <v>107902</v>
+        <v>117602</v>
       </c>
       <c r="Y5" t="n">
-        <v>8474</v>
+        <v>4499</v>
       </c>
       <c r="Z5" t="n">
-        <v>226.78</v>
+        <v>187.23</v>
       </c>
       <c r="AA5" t="n">
-        <v>18385</v>
+        <v>46264</v>
       </c>
       <c r="AB5" t="n">
-        <v>16796</v>
+        <v>46916</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
@@ -1892,88 +1892,88 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45565</v>
+        <v>45747</v>
       </c>
       <c r="B6" t="n">
-        <v>127.65</v>
+        <v>117.79</v>
       </c>
       <c r="C6" t="n">
-        <v>39.56</v>
+        <v>35.43</v>
       </c>
       <c r="D6" t="n">
-        <v>2.53</v>
+        <v>2.82</v>
       </c>
       <c r="E6" t="n">
-        <v>18815</v>
+        <v>32667</v>
       </c>
       <c r="F6" t="n">
-        <v>9.65</v>
+        <v>11</v>
       </c>
       <c r="G6" t="n">
-        <v>7.55</v>
+        <v>6.59</v>
       </c>
       <c r="H6" t="n">
-        <v>1956651330</v>
+        <v>2017326780</v>
       </c>
       <c r="I6" t="n">
-        <v>150634</v>
+        <v>150502</v>
       </c>
       <c r="J6" t="n">
-        <v>88051</v>
+        <v>94565</v>
       </c>
       <c r="K6" t="n">
-        <v>62583</v>
+        <v>55937</v>
       </c>
       <c r="L6" t="n">
-        <v>0.86</v>
+        <v>0.6</v>
       </c>
       <c r="M6" t="n">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="N6" t="n">
-        <v>27.83</v>
+        <v>22.17</v>
       </c>
       <c r="O6" t="n">
-        <v>18.96</v>
+        <v>18.43</v>
       </c>
       <c r="P6" t="n">
-        <v>12.04</v>
+        <v>11.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>690</v>
+        <v>17015</v>
       </c>
       <c r="R6" t="n">
-        <v>5239</v>
+        <v>-29803</v>
       </c>
       <c r="S6" t="n">
-        <v>1732</v>
+        <v>-47</v>
       </c>
       <c r="T6" t="n">
-        <v>-4310</v>
+        <v>-8004</v>
       </c>
       <c r="U6" t="n">
-        <v>5000</v>
+        <v>25019</v>
       </c>
       <c r="V6" t="n">
-        <v>9660</v>
+        <v>19935</v>
       </c>
       <c r="W6" t="n">
-        <v>22245</v>
+        <v>22994</v>
       </c>
       <c r="X6" t="n">
-        <v>95836</v>
+        <v>107902</v>
       </c>
       <c r="Y6" t="n">
-        <v>14315</v>
+        <v>8474</v>
       </c>
       <c r="Z6" t="n">
-        <v>196.54</v>
+        <v>226.78</v>
       </c>
       <c r="AA6" t="n">
-        <v>33174</v>
+        <v>18385</v>
       </c>
       <c r="AB6" t="n">
-        <v>39008</v>
+        <v>16796</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
@@ -1981,88 +1981,88 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45473</v>
+        <v>45565</v>
       </c>
       <c r="B7" t="n">
-        <v>149.71</v>
+        <v>127.65</v>
       </c>
       <c r="C7" t="n">
-        <v>49.42</v>
+        <v>39.56</v>
       </c>
       <c r="D7" t="n">
-        <v>2.02</v>
+        <v>2.53</v>
       </c>
       <c r="E7" t="n">
-        <v>15026</v>
+        <v>18815</v>
       </c>
       <c r="F7" t="n">
-        <v>9.109999999999999</v>
+        <v>9.65</v>
       </c>
       <c r="G7" t="n">
-        <v>8.539999999999999</v>
+        <v>7.55</v>
       </c>
       <c r="H7" t="n">
-        <v>2018882750</v>
+        <v>1956651330</v>
       </c>
       <c r="I7" t="n">
-        <v>150577</v>
+        <v>150634</v>
       </c>
       <c r="J7" t="n">
-        <v>89092</v>
+        <v>88051</v>
       </c>
       <c r="K7" t="n">
-        <v>61485</v>
+        <v>62583</v>
       </c>
       <c r="L7" t="n">
-        <v>0.99</v>
+        <v>0.86</v>
       </c>
       <c r="M7" t="n">
-        <v>0.26</v>
+        <v>0.24</v>
       </c>
       <c r="N7" t="n">
-        <v>33.61</v>
+        <v>27.83</v>
       </c>
       <c r="O7" t="n">
-        <v>17.15</v>
+        <v>18.96</v>
       </c>
       <c r="P7" t="n">
-        <v>10.72</v>
+        <v>12.04</v>
       </c>
       <c r="Q7" t="n">
-        <v>6292</v>
+        <v>690</v>
       </c>
       <c r="R7" t="n">
-        <v>-4276</v>
+        <v>5239</v>
       </c>
       <c r="S7" t="n">
-        <v>-3234</v>
+        <v>1732</v>
       </c>
       <c r="T7" t="n">
-        <v>3597</v>
+        <v>-4310</v>
       </c>
       <c r="U7" t="n">
-        <v>2695</v>
+        <v>5000</v>
       </c>
       <c r="V7" t="n">
-        <v>2846</v>
+        <v>9660</v>
       </c>
       <c r="W7" t="n">
-        <v>22304</v>
+        <v>22245</v>
       </c>
       <c r="X7" t="n">
-        <v>88708</v>
+        <v>95836</v>
       </c>
       <c r="Y7" t="n">
-        <v>15135</v>
+        <v>14315</v>
       </c>
       <c r="Z7" t="n">
-        <v>204.21</v>
+        <v>196.54</v>
       </c>
       <c r="AA7" t="n">
-        <v>21859</v>
+        <v>33174</v>
       </c>
       <c r="AB7" t="n">
-        <v>44292</v>
+        <v>39008</v>
       </c>
       <c r="AC7" t="n">
         <v>0</v>
@@ -2070,88 +2070,88 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45382</v>
+        <v>45473</v>
       </c>
       <c r="B8" t="n">
-        <v>179.72</v>
+        <v>149.71</v>
       </c>
       <c r="C8" t="n">
-        <v>61.56</v>
+        <v>49.42</v>
       </c>
       <c r="D8" t="n">
-        <v>1.62</v>
+        <v>2.02</v>
       </c>
       <c r="E8" t="n">
-        <v>26991</v>
+        <v>15026</v>
       </c>
       <c r="F8" t="n">
-        <v>7.28</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="G8" t="n">
-        <v>8.65</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="H8" t="n">
-        <v>1874689340</v>
+        <v>2018882750</v>
       </c>
       <c r="I8" t="n">
-        <v>153741</v>
+        <v>150577</v>
       </c>
       <c r="J8" t="n">
-        <v>85074</v>
+        <v>89092</v>
       </c>
       <c r="K8" t="n">
-        <v>68667</v>
+        <v>61485</v>
       </c>
       <c r="L8" t="n">
-        <v>1.09</v>
+        <v>0.99</v>
       </c>
       <c r="M8" t="n">
-        <v>0.32</v>
+        <v>0.26</v>
       </c>
       <c r="N8" t="n">
-        <v>30.96</v>
+        <v>33.61</v>
       </c>
       <c r="O8" t="n">
-        <v>13.95</v>
+        <v>17.15</v>
       </c>
       <c r="P8" t="n">
-        <v>8.75</v>
+        <v>10.72</v>
       </c>
       <c r="Q8" t="n">
-        <v>18989</v>
+        <v>6292</v>
       </c>
       <c r="R8" t="n">
-        <v>-17862</v>
+        <v>-4276</v>
       </c>
       <c r="S8" t="n">
-        <v>-1256</v>
+        <v>-3234</v>
       </c>
       <c r="T8" t="n">
-        <v>4064</v>
+        <v>3597</v>
       </c>
       <c r="U8" t="n">
-        <v>14925</v>
+        <v>2695</v>
       </c>
       <c r="V8" t="n">
-        <v>3589</v>
+        <v>2846</v>
       </c>
       <c r="W8" t="n">
-        <v>20424</v>
+        <v>22304</v>
       </c>
       <c r="X8" t="n">
-        <v>87597</v>
+        <v>88708</v>
       </c>
       <c r="Y8" t="n">
-        <v>11024</v>
+        <v>15135</v>
       </c>
       <c r="Z8" t="n">
-        <v>303.53</v>
+        <v>204.21</v>
       </c>
       <c r="AA8" t="n">
-        <v>5618</v>
+        <v>21859</v>
       </c>
       <c r="AB8" t="n">
-        <v>17139</v>
+        <v>44292</v>
       </c>
       <c r="AC8" t="n">
         <v>0</v>
@@ -2159,88 +2159,88 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45199</v>
+        <v>45382</v>
       </c>
       <c r="B9" t="n">
-        <v>132.82</v>
+        <v>179.72</v>
       </c>
       <c r="C9" t="n">
-        <v>57.52</v>
+        <v>61.56</v>
       </c>
       <c r="D9" t="n">
-        <v>1.74</v>
+        <v>1.62</v>
       </c>
       <c r="E9" t="n">
-        <v>11730</v>
+        <v>26991</v>
       </c>
       <c r="F9" t="n">
-        <v>6.9</v>
+        <v>7.28</v>
       </c>
       <c r="G9" t="n">
-        <v>7.17</v>
+        <v>8.65</v>
       </c>
       <c r="H9" t="n">
-        <v>1312132640</v>
+        <v>1874689340</v>
       </c>
       <c r="I9" t="n">
-        <v>153461</v>
+        <v>153741</v>
       </c>
       <c r="J9" t="n">
-        <v>64169</v>
+        <v>85074</v>
       </c>
       <c r="K9" t="n">
-        <v>89292</v>
+        <v>68667</v>
       </c>
       <c r="L9" t="n">
-        <v>2.29</v>
+        <v>1.09</v>
       </c>
       <c r="M9" t="n">
-        <v>0.49</v>
+        <v>0.32</v>
       </c>
       <c r="N9" t="n">
-        <v>36.02</v>
+        <v>30.96</v>
       </c>
       <c r="O9" t="n">
-        <v>12.39</v>
+        <v>13.95</v>
       </c>
       <c r="P9" t="n">
-        <v>6.55</v>
+        <v>8.75</v>
       </c>
       <c r="Q9" t="n">
-        <v>4741</v>
+        <v>18989</v>
       </c>
       <c r="R9" t="n">
-        <v>-2080</v>
+        <v>-17862</v>
       </c>
       <c r="S9" t="n">
-        <v>-2409</v>
+        <v>-1256</v>
       </c>
       <c r="T9" t="n">
-        <v>3717</v>
+        <v>4064</v>
       </c>
       <c r="U9" t="n">
-        <v>1024</v>
+        <v>14925</v>
       </c>
       <c r="V9" t="n">
-        <v>392</v>
+        <v>3589</v>
       </c>
       <c r="W9" t="n">
-        <v>21203</v>
+        <v>20424</v>
       </c>
       <c r="X9" t="n">
-        <v>83461</v>
+        <v>87597</v>
       </c>
       <c r="Y9" t="n">
-        <v>-2219</v>
+        <v>11024</v>
       </c>
       <c r="Z9" t="n">
-        <v>363.25</v>
+        <v>303.53</v>
       </c>
       <c r="AA9" t="n">
-        <v>11786</v>
+        <v>5618</v>
       </c>
       <c r="AB9" t="n">
-        <v>24222</v>
+        <v>17139</v>
       </c>
       <c r="AC9" t="n">
         <v>0</v>
@@ -2248,88 +2248,88 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45107</v>
+        <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>198.63</v>
+        <v>132.82</v>
       </c>
       <c r="C10" t="n">
-        <v>124.15</v>
+        <v>57.52</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8100000000000001</v>
+        <v>1.74</v>
       </c>
       <c r="E10" t="n">
-        <v>8147</v>
+        <v>11730</v>
       </c>
       <c r="F10" t="n">
-        <v>5.02</v>
+        <v>6.9</v>
       </c>
       <c r="G10" t="n">
-        <v>7.95</v>
+        <v>7.17</v>
       </c>
       <c r="H10" t="n">
-        <v>1340752600</v>
+        <v>1312132640</v>
       </c>
       <c r="I10" t="n">
-        <v>153917</v>
+        <v>153461</v>
       </c>
       <c r="J10" t="n">
-        <v>63970</v>
+        <v>64169</v>
       </c>
       <c r="K10" t="n">
-        <v>89947</v>
+        <v>89292</v>
       </c>
       <c r="L10" t="n">
-        <v>2.89</v>
+        <v>2.29</v>
       </c>
       <c r="M10" t="n">
-        <v>0.53</v>
+        <v>0.49</v>
       </c>
       <c r="N10" t="n">
-        <v>45.99</v>
+        <v>36.02</v>
       </c>
       <c r="O10" t="n">
-        <v>6.39</v>
+        <v>12.39</v>
       </c>
       <c r="P10" t="n">
-        <v>5.31</v>
+        <v>6.55</v>
       </c>
       <c r="Q10" t="n">
-        <v>11688</v>
+        <v>4741</v>
       </c>
       <c r="R10" t="n">
-        <v>6133</v>
+        <v>-2080</v>
       </c>
       <c r="S10" t="n">
-        <v>-12893</v>
+        <v>-2409</v>
       </c>
       <c r="T10" t="n">
-        <v>14440</v>
+        <v>3717</v>
       </c>
       <c r="U10" t="n">
-        <v>-2752</v>
+        <v>1024</v>
       </c>
       <c r="V10" t="n">
-        <v>67</v>
+        <v>392</v>
       </c>
       <c r="W10" t="n">
-        <v>21931</v>
+        <v>21203</v>
       </c>
       <c r="X10" t="n">
-        <v>80005</v>
+        <v>83461</v>
       </c>
       <c r="Y10" t="n">
-        <v>-7756</v>
+        <v>-2219</v>
       </c>
       <c r="Z10" t="n">
-        <v>433.45</v>
+        <v>363.25</v>
       </c>
       <c r="AA10" t="n">
-        <v>8349</v>
+        <v>11786</v>
       </c>
       <c r="AB10" t="n">
-        <v>22114</v>
+        <v>24222</v>
       </c>
       <c r="AC10" t="n">
         <v>0</v>
@@ -2337,88 +2337,88 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45016</v>
+        <v>45107</v>
       </c>
       <c r="B11" t="n">
-        <v>333.77</v>
+        <v>198.63</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>124.15</v>
       </c>
       <c r="D11" t="n">
-        <v>-6.93</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>15897</v>
+        <v>8147</v>
       </c>
       <c r="F11" t="n">
-        <v>2.49</v>
+        <v>5.02</v>
       </c>
       <c r="G11" t="n">
-        <v>6.85</v>
+        <v>7.95</v>
       </c>
       <c r="H11" t="n">
-        <v>1058722500</v>
+        <v>1340752600</v>
       </c>
       <c r="I11" t="n">
-        <v>154779</v>
+        <v>153917</v>
       </c>
       <c r="J11" t="n">
-        <v>64405</v>
+        <v>63970</v>
       </c>
       <c r="K11" t="n">
-        <v>90374</v>
+        <v>89947</v>
       </c>
       <c r="L11" t="n">
-        <v>2.54</v>
+        <v>2.89</v>
       </c>
       <c r="M11" t="n">
-        <v>0.58</v>
+        <v>0.53</v>
       </c>
       <c r="N11" t="n">
-        <v>32.27</v>
+        <v>45.99</v>
       </c>
       <c r="O11" t="n">
-        <v>0.11</v>
+        <v>6.39</v>
       </c>
       <c r="P11" t="n">
-        <v>4.96</v>
+        <v>5.31</v>
       </c>
       <c r="Q11" t="n">
-        <v>4788</v>
+        <v>11688</v>
       </c>
       <c r="R11" t="n">
-        <v>-15806</v>
+        <v>6133</v>
       </c>
       <c r="S11" t="n">
-        <v>6354</v>
+        <v>-12893</v>
       </c>
       <c r="T11" t="n">
-        <v>-9419</v>
+        <v>14440</v>
       </c>
       <c r="U11" t="n">
-        <v>14207</v>
+        <v>-2752</v>
       </c>
       <c r="V11" t="n">
-        <v>9258</v>
+        <v>67</v>
       </c>
       <c r="W11" t="n">
-        <v>20450</v>
+        <v>21931</v>
       </c>
       <c r="X11" t="n">
-        <v>82107</v>
+        <v>80005</v>
       </c>
       <c r="Y11" t="n">
-        <v>-11349</v>
+        <v>-7756</v>
       </c>
       <c r="Z11" t="n">
-        <v>653.09</v>
+        <v>433.45</v>
       </c>
       <c r="AA11" t="n">
-        <v>-17708</v>
+        <v>8349</v>
       </c>
       <c r="AB11" t="n">
-        <v>-16253</v>
+        <v>22114</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
@@ -2426,444 +2426,444 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44834</v>
+        <v>45016</v>
       </c>
       <c r="B12" t="n">
-        <v>400.97</v>
+        <v>333.77</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>-1.11</v>
+        <v>-6.93</v>
       </c>
       <c r="E12" t="n">
-        <v>3135</v>
+        <v>15897</v>
       </c>
       <c r="F12" t="n">
-        <v>2.26</v>
+        <v>2.49</v>
       </c>
       <c r="G12" t="n">
-        <v>8.380000000000001</v>
+        <v>6.85</v>
       </c>
       <c r="H12" t="n">
-        <v>1151583000</v>
+        <v>1058722500</v>
       </c>
       <c r="I12" t="n">
-        <v>144580</v>
+        <v>154779</v>
       </c>
       <c r="J12" t="n">
-        <v>58662</v>
+        <v>64405</v>
       </c>
       <c r="K12" t="n">
-        <v>85918</v>
+        <v>90374</v>
       </c>
       <c r="L12" t="n">
-        <v>3.37</v>
+        <v>2.54</v>
       </c>
       <c r="M12" t="n">
-        <v>0.62</v>
+        <v>0.58</v>
       </c>
       <c r="N12" t="n">
-        <v>48.57</v>
+        <v>32.27</v>
       </c>
       <c r="O12" t="n">
         <v>0.11</v>
       </c>
       <c r="P12" t="n">
-        <v>5.39</v>
+        <v>4.96</v>
       </c>
       <c r="Q12" t="n">
-        <v>2439</v>
+        <v>4788</v>
       </c>
       <c r="R12" t="n">
-        <v>-3530</v>
+        <v>-15806</v>
       </c>
       <c r="S12" t="n">
-        <v>-1610</v>
+        <v>6354</v>
       </c>
       <c r="T12" t="n">
-        <v>1785</v>
+        <v>-9419</v>
       </c>
       <c r="U12" t="n">
-        <v>654</v>
+        <v>14207</v>
       </c>
       <c r="V12" t="n">
-        <v>6724</v>
+        <v>9258</v>
       </c>
       <c r="W12" t="n">
-        <v>19485</v>
+        <v>20450</v>
       </c>
       <c r="X12" t="n">
-        <v>73503</v>
+        <v>82107</v>
       </c>
       <c r="Y12" t="n">
-        <v>-8900</v>
+        <v>-11349</v>
       </c>
       <c r="Z12" t="n">
-        <v>457.6</v>
+        <v>653.09</v>
       </c>
       <c r="AA12" t="n">
-        <v>-18014</v>
+        <v>-17708</v>
       </c>
       <c r="AB12" t="n">
-        <v>11259</v>
+        <v>-16253</v>
       </c>
       <c r="AC12" t="n">
-        <v>-3334</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44742</v>
+        <v>44834</v>
       </c>
       <c r="B13" t="n">
-        <v>-532.88</v>
+        <v>400.97</v>
       </c>
       <c r="C13" t="n">
-        <v>7.66</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>13.06</v>
+        <v>-1.11</v>
       </c>
       <c r="E13" t="n">
-        <v>3933</v>
+        <v>3135</v>
       </c>
       <c r="F13" t="n">
-        <v>-1.67</v>
+        <v>2.26</v>
       </c>
       <c r="G13" t="n">
-        <v>8.23</v>
+        <v>8.380000000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>1080686750</v>
+        <v>1151583000</v>
       </c>
       <c r="I13" t="n">
-        <v>142074</v>
+        <v>144580</v>
       </c>
       <c r="J13" t="n">
-        <v>60710</v>
+        <v>58662</v>
       </c>
       <c r="K13" t="n">
-        <v>81364</v>
+        <v>85918</v>
       </c>
       <c r="L13" t="n">
-        <v>2.66</v>
+        <v>3.37</v>
       </c>
       <c r="M13" t="n">
         <v>0.62</v>
       </c>
       <c r="N13" t="n">
-        <v>38.01</v>
+        <v>48.57</v>
       </c>
       <c r="O13" t="n">
-        <v>3.85</v>
+        <v>0.11</v>
       </c>
       <c r="P13" t="n">
-        <v>7.16</v>
+        <v>5.39</v>
       </c>
       <c r="Q13" t="n">
-        <v>11755</v>
+        <v>2439</v>
       </c>
       <c r="R13" t="n">
-        <v>-12984</v>
+        <v>-3530</v>
       </c>
       <c r="S13" t="n">
-        <v>2636</v>
+        <v>-1610</v>
       </c>
       <c r="T13" t="n">
-        <v>10982</v>
+        <v>1785</v>
       </c>
       <c r="U13" t="n">
-        <v>773</v>
+        <v>654</v>
       </c>
       <c r="V13" t="n">
-        <v>8356</v>
+        <v>6724</v>
       </c>
       <c r="W13" t="n">
-        <v>18072</v>
+        <v>19485</v>
       </c>
       <c r="X13" t="n">
-        <v>69521</v>
+        <v>73503</v>
       </c>
       <c r="Y13" t="n">
-        <v>-6624</v>
+        <v>-8900</v>
       </c>
       <c r="Z13" t="n">
-        <v>303.84</v>
+        <v>457.6</v>
       </c>
       <c r="AA13" t="n">
-        <v>15408</v>
+        <v>-18014</v>
       </c>
       <c r="AB13" t="n">
-        <v>16534</v>
+        <v>11259</v>
       </c>
       <c r="AC13" t="n">
-        <v>668</v>
+        <v>-3334</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44651</v>
+        <v>44742</v>
       </c>
       <c r="B14" t="n">
-        <v>-431.67</v>
+        <v>-532.88</v>
       </c>
       <c r="C14" t="n">
-        <v>108.09</v>
+        <v>7.66</v>
       </c>
       <c r="D14" t="n">
-        <v>0.93</v>
+        <v>13.06</v>
       </c>
       <c r="E14" t="n">
-        <v>12647</v>
+        <v>3933</v>
       </c>
       <c r="F14" t="n">
-        <v>-3.3</v>
+        <v>-1.67</v>
       </c>
       <c r="G14" t="n">
-        <v>12.38</v>
+        <v>8.23</v>
       </c>
       <c r="H14" t="n">
-        <v>1659340000</v>
+        <v>1080686750</v>
       </c>
       <c r="I14" t="n">
-        <v>129450</v>
+        <v>142074</v>
       </c>
       <c r="J14" t="n">
-        <v>66385</v>
+        <v>60710</v>
       </c>
       <c r="K14" t="n">
-        <v>63065</v>
+        <v>81364</v>
       </c>
       <c r="L14" t="n">
-        <v>1.47</v>
+        <v>2.66</v>
       </c>
       <c r="M14" t="n">
-        <v>0.47</v>
+        <v>0.62</v>
       </c>
       <c r="N14" t="n">
-        <v>40.04</v>
+        <v>38.01</v>
       </c>
       <c r="O14" t="n">
-        <v>11.34</v>
+        <v>3.85</v>
       </c>
       <c r="P14" t="n">
-        <v>8.48</v>
+        <v>7.16</v>
       </c>
       <c r="Q14" t="n">
-        <v>-2790</v>
+        <v>11755</v>
       </c>
       <c r="R14" t="n">
-        <v>906</v>
+        <v>-12984</v>
       </c>
       <c r="S14" t="n">
-        <v>1990</v>
+        <v>2636</v>
       </c>
       <c r="T14" t="n">
-        <v>-17741</v>
+        <v>10982</v>
       </c>
       <c r="U14" t="n">
-        <v>14951</v>
+        <v>773</v>
       </c>
       <c r="V14" t="n">
-        <v>12773</v>
+        <v>8356</v>
       </c>
       <c r="W14" t="n">
-        <v>14842</v>
+        <v>18072</v>
       </c>
       <c r="X14" t="n">
-        <v>68354</v>
+        <v>69521</v>
       </c>
       <c r="Y14" t="n">
-        <v>-5632</v>
+        <v>-6624</v>
       </c>
       <c r="Z14" t="n">
-        <v>396.01</v>
+        <v>303.84</v>
       </c>
       <c r="AA14" t="n">
-        <v>-15774</v>
+        <v>15408</v>
       </c>
       <c r="AB14" t="n">
-        <v>-14539</v>
+        <v>16534</v>
       </c>
       <c r="AC14" t="n">
-        <v>2666</v>
+        <v>668</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44469</v>
+        <v>44651</v>
       </c>
       <c r="B15" t="n">
-        <v>527.72</v>
+        <v>-431.67</v>
       </c>
       <c r="C15" t="n">
-        <v>65.23999999999999</v>
+        <v>108.09</v>
       </c>
       <c r="D15" t="n">
-        <v>1.53</v>
+        <v>0.93</v>
       </c>
       <c r="E15" t="n">
-        <v>5762</v>
+        <v>12647</v>
       </c>
       <c r="F15" t="n">
-        <v>2.85</v>
+        <v>-3.3</v>
       </c>
       <c r="G15" t="n">
-        <v>13.81</v>
+        <v>12.38</v>
       </c>
       <c r="H15" t="n">
-        <v>1665495000</v>
+        <v>1659340000</v>
       </c>
       <c r="I15" t="n">
-        <v>129528</v>
+        <v>129450</v>
       </c>
       <c r="J15" t="n">
-        <v>78988</v>
+        <v>66385</v>
       </c>
       <c r="K15" t="n">
-        <v>50540</v>
+        <v>63065</v>
       </c>
       <c r="L15" t="n">
-        <v>1.35</v>
+        <v>1.47</v>
       </c>
       <c r="M15" t="n">
-        <v>0.42</v>
+        <v>0.47</v>
       </c>
       <c r="N15" t="n">
-        <v>45.96</v>
+        <v>40.04</v>
       </c>
       <c r="O15" t="n">
-        <v>21.04</v>
+        <v>11.34</v>
       </c>
       <c r="P15" t="n">
-        <v>9.140000000000001</v>
+        <v>8.48</v>
       </c>
       <c r="Q15" t="n">
-        <v>-5402</v>
+        <v>-2790</v>
       </c>
       <c r="R15" t="n">
-        <v>7252</v>
+        <v>906</v>
       </c>
       <c r="S15" t="n">
-        <v>-18419</v>
+        <v>1990</v>
       </c>
       <c r="T15" t="n">
-        <v>-6862</v>
+        <v>-17741</v>
       </c>
       <c r="U15" t="n">
-        <v>1460</v>
+        <v>14951</v>
       </c>
       <c r="V15" t="n">
-        <v>9629</v>
+        <v>12773</v>
       </c>
       <c r="W15" t="n">
-        <v>14380</v>
+        <v>14842</v>
       </c>
       <c r="X15" t="n">
-        <v>61344</v>
+        <v>68354</v>
       </c>
       <c r="Y15" t="n">
-        <v>14537</v>
+        <v>-5632</v>
       </c>
       <c r="Z15" t="n">
-        <v>280.9</v>
+        <v>396.01</v>
       </c>
       <c r="AA15" t="n">
-        <v>-1429</v>
+        <v>-15774</v>
       </c>
       <c r="AB15" t="n">
-        <v>7710</v>
+        <v>-14539</v>
       </c>
       <c r="AC15" t="n">
-        <v>0</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44377</v>
+        <v>44469</v>
       </c>
       <c r="B16" t="n">
-        <v>223.36</v>
+        <v>527.72</v>
       </c>
       <c r="C16" t="n">
-        <v>62.98</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>1.59</v>
+        <v>1.53</v>
       </c>
       <c r="E16" t="n">
-        <v>8232</v>
+        <v>5762</v>
       </c>
       <c r="F16" t="n">
-        <v>6.88</v>
+        <v>2.85</v>
       </c>
       <c r="G16" t="n">
-        <v>15.13</v>
+        <v>13.81</v>
       </c>
       <c r="H16" t="n">
-        <v>1737301000</v>
+        <v>1665495000</v>
       </c>
       <c r="I16" t="n">
-        <v>122390</v>
+        <v>129528</v>
       </c>
       <c r="J16" t="n">
-        <v>89894</v>
+        <v>78988</v>
       </c>
       <c r="K16" t="n">
-        <v>32496</v>
+        <v>50540</v>
       </c>
       <c r="L16" t="n">
-        <v>0.86</v>
+        <v>1.35</v>
       </c>
       <c r="M16" t="n">
-        <v>0.28</v>
+        <v>0.42</v>
       </c>
       <c r="N16" t="n">
-        <v>46.82</v>
+        <v>45.96</v>
       </c>
       <c r="O16" t="n">
-        <v>23.92</v>
+        <v>21.04</v>
       </c>
       <c r="P16" t="n">
-        <v>10.96</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="Q16" t="n">
-        <v>8502</v>
+        <v>-5402</v>
       </c>
       <c r="R16" t="n">
-        <v>-13414</v>
+        <v>7252</v>
       </c>
       <c r="S16" t="n">
-        <v>19119</v>
+        <v>-18419</v>
       </c>
       <c r="T16" t="n">
-        <v>6296</v>
+        <v>-6862</v>
       </c>
       <c r="U16" t="n">
-        <v>2206</v>
+        <v>1460</v>
       </c>
       <c r="V16" t="n">
-        <v>9357</v>
+        <v>9629</v>
       </c>
       <c r="W16" t="n">
-        <v>13871</v>
+        <v>14380</v>
       </c>
       <c r="X16" t="n">
-        <v>57080</v>
+        <v>61344</v>
       </c>
       <c r="Y16" t="n">
-        <v>23056</v>
+        <v>14537</v>
       </c>
       <c r="Z16" t="n">
-        <v>193.31</v>
+        <v>280.9</v>
       </c>
       <c r="AA16" t="n">
-        <v>38394</v>
+        <v>-1429</v>
       </c>
       <c r="AB16" t="n">
-        <v>23201</v>
+        <v>7710</v>
       </c>
       <c r="AC16" t="n">
         <v>0</v>
@@ -2871,90 +2871,179 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
+        <v>44377</v>
+      </c>
+      <c r="B17" t="n">
+        <v>223.36</v>
+      </c>
+      <c r="C17" t="n">
+        <v>62.98</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="E17" t="n">
+        <v>8232</v>
+      </c>
+      <c r="F17" t="n">
+        <v>6.88</v>
+      </c>
+      <c r="G17" t="n">
+        <v>15.13</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1737301000</v>
+      </c>
+      <c r="I17" t="n">
+        <v>122390</v>
+      </c>
+      <c r="J17" t="n">
+        <v>89894</v>
+      </c>
+      <c r="K17" t="n">
+        <v>32496</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="N17" t="n">
+        <v>46.82</v>
+      </c>
+      <c r="O17" t="n">
+        <v>23.92</v>
+      </c>
+      <c r="P17" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>8502</v>
+      </c>
+      <c r="R17" t="n">
+        <v>-13414</v>
+      </c>
+      <c r="S17" t="n">
+        <v>19119</v>
+      </c>
+      <c r="T17" t="n">
+        <v>6296</v>
+      </c>
+      <c r="U17" t="n">
+        <v>2206</v>
+      </c>
+      <c r="V17" t="n">
+        <v>9357</v>
+      </c>
+      <c r="W17" t="n">
+        <v>13871</v>
+      </c>
+      <c r="X17" t="n">
+        <v>57080</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>23056</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>193.31</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>38394</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>23201</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>44286</v>
       </c>
-      <c r="B17" t="n">
+      <c r="B18" t="n">
         <v>192.35</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C18" t="n">
         <v>69.83</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>1.43</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>16373</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>7.47</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G18" t="n">
         <v>15.09</v>
       </c>
-      <c r="H17" t="n">
+      <c r="H18" t="n">
         <v>1559376000</v>
       </c>
-      <c r="I17" t="n">
+      <c r="I18" t="n">
         <v>100794</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J18" t="n">
         <v>73270</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K18" t="n">
         <v>27524</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L18" t="n">
         <v>0.71</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M18" t="n">
         <v>0.27</v>
       </c>
-      <c r="N17" t="n">
+      <c r="N18" t="n">
         <v>40.77</v>
       </c>
-      <c r="O17" t="n">
+      <c r="O18" t="n">
         <v>21.5</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>10.98</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q18" t="n">
         <v>4213</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R18" t="n">
         <v>-8666</v>
       </c>
-      <c r="S17" t="n">
+      <c r="S18" t="n">
         <v>-3476</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T18" t="n">
         <v>-7869</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U18" t="n">
         <v>12082</v>
       </c>
-      <c r="V17" t="n">
+      <c r="V18" t="n">
         <v>9114</v>
       </c>
-      <c r="W17" t="n">
+      <c r="W18" t="n">
         <v>12488</v>
       </c>
-      <c r="X17" t="n">
+      <c r="X18" t="n">
         <v>52291</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Y18" t="n">
         <v>6004</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="Z18" t="n">
         <v>288.2</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AA18" t="n">
         <v>-6761</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB18" t="n">
         <v>-1731</v>
       </c>
-      <c r="AC17" t="n">
+      <c r="AC18" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>